<commit_message>
Nuevo correo y avances errores ortograficos
</commit_message>
<xml_diff>
--- a/data/ChedrahuiQA_Lexico.xlsx
+++ b/data/ChedrahuiQA_Lexico.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atcon\Desktop\Playwright\playwright-piloto2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE7D5B76-ED80-41E4-9F9B-22517A3CAAD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB33C48-CC10-471F-91B6-10A8B1FCC92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Long Tail" sheetId="6" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="129">
   <si>
     <t>Término</t>
   </si>
@@ -158,9 +158,6 @@
     <t>yoghurt</t>
   </si>
   <si>
-    <t>desodorante, antitranspirante</t>
-  </si>
-  <si>
     <t>jabón, shampoo, acondicionador, papel higiénico, pasta dental, cepillo dental, hilo dental, enjuague bucal, cotonetes, crema corporal</t>
   </si>
   <si>
@@ -183,9 +180,6 @@
   </si>
   <si>
     <t>huevos, yogurt griego, pechuga de pollo, atún en lata, proteína en polvo, claras de huevo pasteurizadas</t>
-  </si>
-  <si>
-    <t>lavadora, centro de lavado</t>
   </si>
   <si>
     <t>mascarilla capilar, acondicionador, aceite capilar, serum capilar, keratina, tratamiento leave-in, iggkjhkjh</t>
@@ -356,15 +350,6 @@
     <t>Pampers, KleenBebé</t>
   </si>
   <si>
-    <t>pañales, pañal</t>
-  </si>
-  <si>
-    <t>refrigerador, nevera</t>
-  </si>
-  <si>
-    <t>papel Higiénico, papel de baño</t>
-  </si>
-  <si>
     <t>piña</t>
   </si>
   <si>
@@ -457,6 +442,18 @@
   </si>
   <si>
     <t>Mostrar listado de los resultados que no tengan</t>
+  </si>
+  <si>
+    <t>papel Higiénico</t>
+  </si>
+  <si>
+    <t>desodorante</t>
+  </si>
+  <si>
+    <t>pañales</t>
+  </si>
+  <si>
+    <t>lavadora</t>
   </si>
 </sst>
 </file>
@@ -612,13 +609,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -969,156 +966,156 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" t="s">
         <v>71</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" t="s">
         <v>72</v>
       </c>
-      <c r="C2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>74</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" s="13" t="s">
         <v>76</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="13"/>
+        <v>45</v>
+      </c>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="G4" s="13"/>
+        <v>46</v>
+      </c>
+      <c r="G4" s="14"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="G5" s="13"/>
+        <v>47</v>
+      </c>
+      <c r="G5" s="14"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="G6" s="13"/>
+        <v>48</v>
+      </c>
+      <c r="G6" s="14"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="13"/>
+        <v>49</v>
+      </c>
+      <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" s="13"/>
+        <v>50</v>
+      </c>
+      <c r="G8" s="14"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="13"/>
+        <v>51</v>
+      </c>
+      <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="G10" s="13"/>
+        <v>52</v>
+      </c>
+      <c r="G10" s="14"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="G11" s="13"/>
+        <v>53</v>
+      </c>
+      <c r="G11" s="14"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G12" s="9"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G13" s="9"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G16" s="9"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G17" s="9"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G18" s="9"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1146,16 +1143,16 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>81</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -1168,67 +1165,67 @@
     </row>
     <row r="2" spans="1:12" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
         <v>82</v>
       </c>
-      <c r="C2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>85</v>
+      <c r="D2" s="14" t="s">
+        <v>83</v>
       </c>
       <c r="L2"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>116</v>
-      </c>
-      <c r="D3" s="13"/>
+        <v>111</v>
+      </c>
+      <c r="D3" s="14"/>
       <c r="L3"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="D4" s="13"/>
+      <c r="D4" s="14"/>
       <c r="L4"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="D5" s="13"/>
+      <c r="D5" s="14"/>
       <c r="L5"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="D6" s="13"/>
+      <c r="D6" s="14"/>
       <c r="L6"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="D7" s="13"/>
+      <c r="D7" s="14"/>
       <c r="L7"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="D8" s="14"/>
+      <c r="D8" s="12"/>
       <c r="L8"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>117</v>
+      <c r="D9" s="12" t="s">
+        <v>112</v>
       </c>
       <c r="L9"/>
     </row>
@@ -1349,8 +1346,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="63.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1359,13 +1356,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1376,10 +1373,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>118</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>105</v>
+        <v>113</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1387,51 +1384,51 @@
         <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
-      </c>
-      <c r="D3" s="13"/>
+        <v>125</v>
+      </c>
+      <c r="D3" s="14"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="13"/>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="13"/>
+        <v>126</v>
+      </c>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D6" s="13"/>
+        <v>95</v>
+      </c>
+      <c r="D6" s="14"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="13"/>
+        <v>128</v>
+      </c>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -1440,7 +1437,7 @@
       <c r="B8" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="13"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -1450,9 +1447,9 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>119</v>
-      </c>
-      <c r="D9" s="13"/>
+        <v>114</v>
+      </c>
+      <c r="D9" s="14"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -1462,16 +1459,16 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
-      </c>
-      <c r="D10" s="13"/>
+        <v>98</v>
+      </c>
+      <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C11" t="s">
         <v>10</v>
@@ -1479,24 +1476,24 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
         <v>13</v>
@@ -1504,24 +1501,24 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1551,19 +1548,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1571,65 +1568,65 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F2" s="13" t="s">
         <v>109</v>
-      </c>
-      <c r="C2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D2" t="s">
-        <v>110</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="D3" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="13"/>
+      <c r="F3" s="14"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="13"/>
+      <c r="F4" s="14"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="13"/>
+      <c r="F5" s="14"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="13"/>
+      <c r="F6" s="14"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="13"/>
+      <c r="F7" s="14"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="13"/>
+      <c r="F8" s="14"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -1639,10 +1636,10 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -1681,7 +1678,7 @@
         <v>16</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1689,7 +1686,7 @@
         <v>17</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1697,7 +1694,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -1705,7 +1702,7 @@
         <v>19</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -1713,7 +1710,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1721,7 +1718,7 @@
         <v>21</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -1729,7 +1726,7 @@
         <v>22</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -1737,7 +1734,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -1745,7 +1742,7 @@
         <v>24</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1764,32 +1761,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Inclusion empathy resultados vacios
</commit_message>
<xml_diff>
--- a/data/ChedrahuiQA_Lexico.xlsx
+++ b/data/ChedrahuiQA_Lexico.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atcon\Desktop\Playwright\playwright-piloto2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7985E4C1-95CC-4A88-AE03-C2A7B5939B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A33C558-E634-4164-BA54-383B311E57D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Long Tail" sheetId="6" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errores Ortográficos'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Frecuencia Alta'!$A$1:$A$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Long Tail'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resultados Vacíos'!$A$1:$L$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resultados Vacíos'!$A$1:$L$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Semánticos!$A$1:$C$1</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -48,12 +48,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="125">
   <si>
     <t>Término</t>
   </si>
   <si>
     <t>shampoo</t>
+  </si>
+  <si>
+    <t>papel higiénico</t>
+  </si>
+  <si>
+    <t>cafe</t>
+  </si>
+  <si>
+    <t>leche</t>
   </si>
   <si>
     <t>galletas</t>
@@ -211,189 +220,230 @@
     <t>Termino</t>
   </si>
   <si>
-    <t xml:space="preserve">Relevancia </t>
-  </si>
-  <si>
     <t>Funcionalidad</t>
   </si>
   <si>
-    <t>Relacion 1, Relacion 2, Relacion 3, Relacion 4</t>
-  </si>
-  <si>
     <t>Parcialmente Relevantes</t>
   </si>
   <si>
-    <t>Parcial 1, Parcial 2, Parcial 3</t>
-  </si>
-  <si>
-    <t>Se buscan los 25 terminos en buscador actual.
+    <t>uevo blanc</t>
+  </si>
+  <si>
+    <t>huevo blanco</t>
+  </si>
+  <si>
+    <t>gayetas de arros</t>
+  </si>
+  <si>
+    <t>galletas de arroz</t>
+  </si>
+  <si>
+    <t>coca 2</t>
+  </si>
+  <si>
+    <t>coca cola 2 litros</t>
+  </si>
+  <si>
+    <t>vino rozado</t>
+  </si>
+  <si>
+    <t>vino rosado</t>
+  </si>
+  <si>
+    <t>Correccion</t>
+  </si>
+  <si>
+    <t>Pampers, KleenBebé</t>
+  </si>
+  <si>
+    <t>piña</t>
+  </si>
+  <si>
+    <t>vino</t>
+  </si>
+  <si>
+    <t>ariel</t>
+  </si>
+  <si>
+    <t>Reglas</t>
+  </si>
+  <si>
+    <t>CC=Si se muestra corrección en el campo de búsqueda y productos relacionados.
+CP=Se muestra correccion en la busqueda, pero no se encuentra similitudes de resultados pero si equivalencia.
+SR=No muestra corrección en busqueda, devuelve algunos productos en equivalencia.
+SN=No corrige y sin resultados</t>
+  </si>
+  <si>
+    <t>Mismo universo diferente intencion</t>
+  </si>
+  <si>
+    <t>Categoria y atributo clave</t>
+  </si>
+  <si>
+    <t>Atributo secundario</t>
+  </si>
+  <si>
+    <t>Reporte que por cada resultado se evalue.
+Si se coincide con categoria y Marca = 3
+Si se coincide con categoria pero distinto atributo sin coincidir con secundario = 2
+Sin coincidencias Categoria y atributo clave, marca, atributo secundario, pero si con mismo universo = 1
+Sin coincidencias con ninguno de las columnas = 0</t>
+  </si>
+  <si>
+    <t>jabon para cabello</t>
+  </si>
+  <si>
+    <t>Tequila</t>
+  </si>
+  <si>
+    <t>Notas:</t>
+  </si>
+  <si>
+    <t>Evaluar resultados si tienen o no imagen</t>
+  </si>
+  <si>
+    <t>En cada reporte indicar numero de resultados por cada calificacion, los de codigo de letra o numero según aplique</t>
+  </si>
+  <si>
+    <t>En errores ortograficos mostrar listado de los resultados de busqueda que no coinciden con las palabras corregidas para detectar errores en carga producto</t>
+  </si>
+  <si>
+    <t>Todas las pruebas seran en tienda polanco</t>
+  </si>
+  <si>
+    <t>Mostrar listado de los resultados que no tengan</t>
+  </si>
+  <si>
+    <t>papel Higiénico</t>
+  </si>
+  <si>
+    <t>desodorante</t>
+  </si>
+  <si>
+    <t>pañales</t>
+  </si>
+  <si>
+    <t>lavadora</t>
+  </si>
+  <si>
+    <t>piña en almibar</t>
+  </si>
+  <si>
+    <t>pina en almivar</t>
+  </si>
+  <si>
+    <t>Alpura</t>
+  </si>
+  <si>
+    <t>1L, 1 litro, light, descremada</t>
+  </si>
+  <si>
+    <t>yogurt bebible</t>
+  </si>
+  <si>
+    <t>pañales huggies etapa 4</t>
+  </si>
+  <si>
+    <t>Huggies</t>
+  </si>
+  <si>
+    <t>40 piezas, jumbo, para bebé, talla 4</t>
+  </si>
+  <si>
+    <t>toallitas húmedas</t>
+  </si>
+  <si>
+    <t>café soluble nescafé clásico 200g</t>
+  </si>
+  <si>
+    <t>Nescafé</t>
+  </si>
+  <si>
+    <t>200g, frasco, clásico, instantáneo</t>
+  </si>
+  <si>
+    <t>crema para café</t>
+  </si>
+  <si>
+    <t>leche deslactosada alpura 1L</t>
+  </si>
+  <si>
+    <t>leche, deslactosada</t>
+  </si>
+  <si>
+    <t>pañales, etapa, 4</t>
+  </si>
+  <si>
+    <t>café, soluble</t>
+  </si>
+  <si>
+    <t>poquemon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se buscan los 25 terminos en buscador actual.
 Se buscan los 25 terminos en buscador empathy.
 Se muestran los resultados de los terminos que si tienen resultados relevantes en buscador actual.
 De los que no se muestra un listado con atributo R, P, V, I segun lo siguiente:
 R= Resultado relevante
 P=Resultados sin similitudes Relevantes pero con palabnras en relevantes.
 V= 0 Resultados en Empathy
-I = Resultados pero sin coincidencias con Relevantes ni Parcialmente</t>
-  </si>
-  <si>
-    <t>uevo blanc</t>
-  </si>
-  <si>
-    <t>huevo blanco</t>
-  </si>
-  <si>
-    <t>gayetas de arros</t>
-  </si>
-  <si>
-    <t>galletas de arroz</t>
-  </si>
-  <si>
-    <t>coca 2</t>
-  </si>
-  <si>
-    <t>coca cola 2 litros</t>
-  </si>
-  <si>
-    <t>vino rozado</t>
-  </si>
-  <si>
-    <t>vino rosado</t>
-  </si>
-  <si>
-    <t>Correccion</t>
-  </si>
-  <si>
-    <t>Pampers, KleenBebé</t>
-  </si>
-  <si>
-    <t>piña</t>
-  </si>
-  <si>
-    <t>vino</t>
-  </si>
-  <si>
-    <t>ariel</t>
-  </si>
-  <si>
-    <t>Reglas</t>
-  </si>
-  <si>
-    <t>CC=Si se muestra corrección en el campo de búsqueda y productos relacionados.
-CP=Se muestra correccion en la busqueda, pero no se encuentra similitudes de resultados pero si equivalencia.
-SR=No muestra corrección en busqueda, devuelve algunos productos en equivalencia.
-SN=No corrige y sin resultados</t>
-  </si>
-  <si>
-    <t>Mismo universo diferente intencion</t>
-  </si>
-  <si>
-    <t>Categoria y atributo clave</t>
-  </si>
-  <si>
-    <t>Atributo secundario</t>
-  </si>
-  <si>
-    <t>Reporte que por cada resultado se evalue.
-Si se coincide con categoria y Marca = 3
-Si se coincide con categoria pero distinto atributo sin coincidir con secundario = 2
-Sin coincidencias Categoria y atributo clave, marca, atributo secundario, pero si con mismo universo = 1
-Sin coincidencias con ninguno de las columnas = 0</t>
-  </si>
-  <si>
-    <t>busqueda 1</t>
-  </si>
-  <si>
-    <t>busqueda 2</t>
-  </si>
-  <si>
-    <t>Conteo de resultados y especificacion si son R, P o I</t>
-  </si>
-  <si>
-    <t>jabon para cabello</t>
-  </si>
-  <si>
-    <t>Tequila</t>
-  </si>
-  <si>
-    <t>Notas:</t>
-  </si>
-  <si>
-    <t>Evaluar resultados si tienen o no imagen</t>
-  </si>
-  <si>
-    <t>En cada reporte indicar numero de resultados por cada calificacion, los de codigo de letra o numero según aplique</t>
-  </si>
-  <si>
-    <t>En errores ortograficos mostrar listado de los resultados de busqueda que no coinciden con las palabras corregidas para detectar errores en carga producto</t>
-  </si>
-  <si>
-    <t>Todas las pruebas seran en tienda polanco</t>
-  </si>
-  <si>
-    <t>Mostrar listado de los resultados que no tengan</t>
-  </si>
-  <si>
-    <t>papel Higiénico</t>
-  </si>
-  <si>
-    <t>desodorante</t>
-  </si>
-  <si>
-    <t>pañales</t>
-  </si>
-  <si>
-    <t>lavadora</t>
-  </si>
-  <si>
-    <t>piña en almibar</t>
-  </si>
-  <si>
-    <t>pina en almivar</t>
-  </si>
-  <si>
-    <t>Alpura</t>
-  </si>
-  <si>
-    <t>1L, 1 litro, light, descremada</t>
-  </si>
-  <si>
-    <t>yogurt bebible</t>
-  </si>
-  <si>
-    <t>pañales huggies etapa 4</t>
-  </si>
-  <si>
-    <t>Huggies</t>
-  </si>
-  <si>
-    <t>40 piezas, jumbo, para bebé, talla 4</t>
-  </si>
-  <si>
-    <t>toallitas húmedas</t>
-  </si>
-  <si>
-    <t>café soluble nescafé clásico 200g</t>
-  </si>
-  <si>
-    <t>Nescafé</t>
-  </si>
-  <si>
-    <t>200g, frasco, clásico, instantáneo</t>
-  </si>
-  <si>
-    <t>crema para café</t>
-  </si>
-  <si>
-    <t>leche deslactosada alpura 1L</t>
-  </si>
-  <si>
-    <t>leche, deslactosada</t>
-  </si>
-  <si>
-    <t>pañales, etapa, 4</t>
-  </si>
-  <si>
-    <t>café, soluble</t>
+I = Resultados pero sin coincidencias con Relevantes ni Parcialmente
+Conteo de resultados y especificacion si son R, P o I
+</t>
+  </si>
+  <si>
+    <t>pokemon</t>
+  </si>
+  <si>
+    <t>pikachu</t>
+  </si>
+  <si>
+    <t>Pokemon, Pocket Monster, Pokémon</t>
+  </si>
+  <si>
+    <t>Pikachu, Eevee, Lapras</t>
+  </si>
+  <si>
+    <t>Relevancia</t>
+  </si>
+  <si>
+    <t>juguetes</t>
+  </si>
+  <si>
+    <t>jitomate</t>
+  </si>
+  <si>
+    <t>barbie</t>
+  </si>
+  <si>
+    <t>tomate</t>
+  </si>
+  <si>
+    <t>fabuloso</t>
+  </si>
+  <si>
+    <t>saba</t>
+  </si>
+  <si>
+    <t>chuleta de cerdo</t>
+  </si>
+  <si>
+    <t>mayonesa</t>
+  </si>
+  <si>
+    <t>pantene</t>
+  </si>
+  <si>
+    <t>tecnologia</t>
+  </si>
+  <si>
+    <t>aceite</t>
+  </si>
+  <si>
+    <t>cereal</t>
+  </si>
+  <si>
+    <t>suavitel</t>
   </si>
 </sst>
 </file>
@@ -516,7 +566,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -527,6 +576,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -882,45 +934,45 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -933,7 +985,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07CF1A1E-23EA-440E-B96D-E9DFBACBA6A8}">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
@@ -945,16 +997,16 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>52</v>
+        <v>111</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -967,184 +1019,28 @@
     </row>
     <row r="2" spans="1:12" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>109</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>57</v>
+        <v>110</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>106</v>
       </c>
       <c r="L2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="10"/>
-      <c r="L3"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="D4" s="10"/>
-      <c r="L4"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="D5" s="10"/>
-      <c r="L5"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="D6" s="10"/>
-      <c r="L6"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="D7" s="10"/>
-      <c r="L7"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="D8" s="8"/>
-      <c r="L8"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="L9"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="L10"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="L11"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="L12"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="L13"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="L14"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="L15"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="L16"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="L17"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="L18"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="L19"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="L20"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="L21"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="L22"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="L23"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="L24"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="L25"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="L26"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L26" xr:uid="{07CF1A1E-23EA-440E-B96D-E9DFBACBA6A8}"/>
-  <mergeCells count="1">
-    <mergeCell ref="D2:D7"/>
-  </mergeCells>
+  <autoFilter ref="A1:L2" xr:uid="{07CF1A1E-23EA-440E-B96D-E9DFBACBA6A8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A479586D-24F4-4D87-B01B-4E29F29415E8}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.88671875" bestFit="1" customWidth="1"/>
@@ -1158,166 +1054,177 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>72</v>
+        <v>76</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D3" s="10"/>
+        <v>84</v>
+      </c>
+      <c r="D3" s="9"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="10"/>
+        <v>11</v>
+      </c>
+      <c r="D4" s="9"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
-      </c>
-      <c r="D5" s="10"/>
+        <v>85</v>
+      </c>
+      <c r="D5" s="9"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="10"/>
+        <v>66</v>
+      </c>
+      <c r="D6" s="9"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
-      </c>
-      <c r="D7" s="10"/>
+        <v>87</v>
+      </c>
+      <c r="D7" s="9"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="10"/>
+        <v>31</v>
+      </c>
+      <c r="D8" s="9"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="D9" s="9"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="10"/>
+        <v>69</v>
+      </c>
+      <c r="D10" s="9"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
         <v>58</v>
       </c>
-      <c r="B11" t="s">
-        <v>59</v>
-      </c>
       <c r="C11" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" t="s">
         <v>60</v>
       </c>
-      <c r="B12" t="s">
-        <v>61</v>
-      </c>
       <c r="C12" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" t="s">
         <v>62</v>
       </c>
-      <c r="B13" t="s">
-        <v>63</v>
-      </c>
       <c r="C13" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" t="s">
         <v>64</v>
       </c>
-      <c r="B14" t="s">
-        <v>65</v>
-      </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" t="s">
+        <v>107</v>
+      </c>
+      <c r="C16" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1331,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
@@ -1347,76 +1254,201 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="11" t="s">
+    </row>
+    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D3" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E3" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="F2" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="F3" s="13"/>
+    </row>
+    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C3" s="11" t="s">
+      <c r="B4" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="F3" s="13"/>
-    </row>
-    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>104</v>
-      </c>
       <c r="F4" s="13"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" s="10" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
+        <v>124</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:A4" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
@@ -1441,79 +1473,79 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1532,32 +1564,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajustes listos de alta frecuencia
</commit_message>
<xml_diff>
--- a/data/ChedrahuiQA_Lexico.xlsx
+++ b/data/ChedrahuiQA_Lexico.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atcon\Desktop\Playwright\playwright-piloto2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A33C558-E634-4164-BA54-383B311E57D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C400F9B-B9D4-42E0-A6C7-FF90A0E6D435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Long Tail" sheetId="6" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errores Ortográficos'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Frecuencia Alta'!$A$1:$A$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Frecuencia Alta'!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Long Tail'!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resultados Vacíos'!$A$1:$L$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Semánticos!$A$1:$C$1</definedName>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="170">
   <si>
     <t>Término</t>
   </si>
@@ -57,9 +57,6 @@
   </si>
   <si>
     <t>papel higiénico</t>
-  </si>
-  <si>
-    <t>cafe</t>
   </si>
   <si>
     <t>leche</t>
@@ -274,22 +271,6 @@
 SN=No corrige y sin resultados</t>
   </si>
   <si>
-    <t>Mismo universo diferente intencion</t>
-  </si>
-  <si>
-    <t>Categoria y atributo clave</t>
-  </si>
-  <si>
-    <t>Atributo secundario</t>
-  </si>
-  <si>
-    <t>Reporte que por cada resultado se evalue.
-Si se coincide con categoria y Marca = 3
-Si se coincide con categoria pero distinto atributo sin coincidir con secundario = 2
-Sin coincidencias Categoria y atributo clave, marca, atributo secundario, pero si con mismo universo = 1
-Sin coincidencias con ninguno de las columnas = 0</t>
-  </si>
-  <si>
     <t>jabon para cabello</t>
   </si>
   <si>
@@ -332,24 +313,12 @@
     <t>pina en almivar</t>
   </si>
   <si>
-    <t>Alpura</t>
-  </si>
-  <si>
-    <t>1L, 1 litro, light, descremada</t>
-  </si>
-  <si>
-    <t>yogurt bebible</t>
-  </si>
-  <si>
     <t>pañales huggies etapa 4</t>
   </si>
   <si>
     <t>Huggies</t>
   </si>
   <si>
-    <t>40 piezas, jumbo, para bebé, talla 4</t>
-  </si>
-  <si>
     <t>toallitas húmedas</t>
   </si>
   <si>
@@ -359,16 +328,7 @@
     <t>Nescafé</t>
   </si>
   <si>
-    <t>200g, frasco, clásico, instantáneo</t>
-  </si>
-  <si>
     <t>crema para café</t>
-  </si>
-  <si>
-    <t>leche deslactosada alpura 1L</t>
-  </si>
-  <si>
-    <t>leche, deslactosada</t>
   </si>
   <si>
     <t>pañales, etapa, 4</t>
@@ -434,9 +394,6 @@
     <t>pantene</t>
   </si>
   <si>
-    <t>tecnologia</t>
-  </si>
-  <si>
     <t>aceite</t>
   </si>
   <si>
@@ -444,13 +401,189 @@
   </si>
   <si>
     <t>suavitel</t>
+  </si>
+  <si>
+    <t>200g</t>
+  </si>
+  <si>
+    <t>clásico, instantáneo, frasco</t>
+  </si>
+  <si>
+    <t>40 piezas, 40 unidades</t>
+  </si>
+  <si>
+    <t>jumbo, para bebé, talla 4, bebe</t>
+  </si>
+  <si>
+    <t>Relacionados</t>
+  </si>
+  <si>
+    <t>jitomate, tomate</t>
+  </si>
+  <si>
+    <t>infantil, ropa de niño, ropa para niño</t>
+  </si>
+  <si>
+    <t>Si existe al menos una equivalencia true = 2
+Si equivalencia false pero al menos un relacion true = 1
+Si Equivalencia &amp; Relacionado false = 0</t>
+  </si>
+  <si>
+    <t>papel higiénico, papel de baño</t>
+  </si>
+  <si>
+    <t>pasta de dientes, toalla, servilletas</t>
+  </si>
+  <si>
+    <t>acondicionador, gel para cabello, crema para peinar</t>
+  </si>
+  <si>
+    <t>barbie, muñeca, muñeca de juguete</t>
+  </si>
+  <si>
+    <t>tomate, jitomate</t>
+  </si>
+  <si>
+    <t>suavizante, cloro, quitamanchas</t>
+  </si>
+  <si>
+    <t>leche, leche entera, leche deslactosada</t>
+  </si>
+  <si>
+    <t>yogur, queso, crema</t>
+  </si>
+  <si>
+    <t>refrigerador, refri, nevera</t>
+  </si>
+  <si>
+    <t>congelador, horno de microondas, estufa</t>
+  </si>
+  <si>
+    <t>desodorante, antitranspirante</t>
+  </si>
+  <si>
+    <t>perfume, gel de baño, crema corporal</t>
+  </si>
+  <si>
+    <t>galletas, galletas dulces, galletas saladas</t>
+  </si>
+  <si>
+    <t>pan, cereal, botanas</t>
+  </si>
+  <si>
+    <t>secadora, detergente, suavizante</t>
+  </si>
+  <si>
+    <t>pañales, pañales desechables</t>
+  </si>
+  <si>
+    <t>cerveza, cerveza clara, cerveza oscura</t>
+  </si>
+  <si>
+    <t>botanas, vino, refresco</t>
+  </si>
+  <si>
+    <t>huevo, huevo blanco, huevo rojo</t>
+  </si>
+  <si>
+    <t>leche, mantequilla, queso</t>
+  </si>
+  <si>
+    <t>chuleta de cerdo, carne de cerdo</t>
+  </si>
+  <si>
+    <t>res, pollo, tocino</t>
+  </si>
+  <si>
+    <t>mayonesa, aderezo</t>
+  </si>
+  <si>
+    <t>mostaza, ketchup, salsa</t>
+  </si>
+  <si>
+    <t>acondicionador, tratamiento capilar, crema para peinar</t>
+  </si>
+  <si>
+    <t>aceite, aceite vegetal, aceite de cocina</t>
+  </si>
+  <si>
+    <t>manteca, mantequilla, vinagre</t>
+  </si>
+  <si>
+    <t>cereal, cereal de desayuno</t>
+  </si>
+  <si>
+    <t>leche, avena, granola</t>
+  </si>
+  <si>
+    <t>detergente, cloro, aromatizante de ropa</t>
+  </si>
+  <si>
+    <t>shampoo, champú, jabón para cabello</t>
+  </si>
+  <si>
+    <t>juguetes, casa de muñecas, accesorios de muñeca</t>
+  </si>
+  <si>
+    <t>tomatillo, puré de tomate, salsa de tomate</t>
+  </si>
+  <si>
+    <t>ariel, detergente, jabón para ropa</t>
+  </si>
+  <si>
+    <t>café</t>
+  </si>
+  <si>
+    <t>café, café molido, café soluble</t>
+  </si>
+  <si>
+    <t>azúcar, crema para café, té</t>
+  </si>
+  <si>
+    <t>fabuloso, limpiador líquido, limpiador multiusos</t>
+  </si>
+  <si>
+    <t>desinfectante, cloro, detergente líquido</t>
+  </si>
+  <si>
+    <t>saba, toallas femeninas, toallas sanitarias</t>
+  </si>
+  <si>
+    <t>tampones, pantiprotector, papel higiénico</t>
+  </si>
+  <si>
+    <t>lavadora, máquina de lavar</t>
+  </si>
+  <si>
+    <t>toallitas húmedas, leche infantil, biberón</t>
+  </si>
+  <si>
+    <t>pantene, shampoo, champú, cuidado del cabello</t>
+  </si>
+  <si>
+    <t>tecnología</t>
+  </si>
+  <si>
+    <t>suavitel, suavizante, suavizante de telas</t>
+  </si>
+  <si>
+    <t>juguetes, juguete, juego de mesa, carro control remoto, muñeca, peluche, vehículo</t>
+  </si>
+  <si>
+    <t>tomatillo, puré de tomate, sopa de tomate, catsup, ketchup</t>
+  </si>
+  <si>
+    <t>tecnología, electrónica, celular, computadora, pantalla, televisor, celular, movil, consola, dvd, laptop</t>
+  </si>
+  <si>
+    <t>batería, pilas, extensión</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -460,6 +593,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -555,7 +696,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -564,8 +705,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -918,13 +1060,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28555630-8AA8-4C83-B7EB-C61073BD67A5}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.21875" customWidth="1"/>
     <col min="4" max="4" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="66.109375" customWidth="1"/>
     <col min="7" max="7" width="23.6640625" customWidth="1"/>
   </cols>
@@ -934,50 +1076,93 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="12" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>53</v>
-      </c>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="E3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D8" s="6"/>
     </row>
   </sheetData>
   <autoFilter ref="A1" xr:uid="{28555630-8AA8-4C83-B7EB-C61073BD67A5}"/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -997,16 +1182,16 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -1019,16 +1204,16 @@
     </row>
     <row r="2" spans="1:12" ht="172.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>106</v>
+        <v>98</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>94</v>
       </c>
       <c r="L2"/>
     </row>
@@ -1054,177 +1239,177 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="8" t="s">
         <v>71</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D3" s="9"/>
+        <v>79</v>
+      </c>
+      <c r="D3" s="10"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="9"/>
+        <v>10</v>
+      </c>
+      <c r="D4" s="10"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D5" s="9"/>
+        <v>80</v>
+      </c>
+      <c r="D5" s="10"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" s="9"/>
+        <v>65</v>
+      </c>
+      <c r="D6" s="10"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>87</v>
-      </c>
-      <c r="D7" s="9"/>
+        <v>82</v>
+      </c>
+      <c r="D7" s="10"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="9"/>
+        <v>30</v>
+      </c>
+      <c r="D8" s="10"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D9" s="9"/>
+        <v>72</v>
+      </c>
+      <c r="D9" s="10"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>69</v>
-      </c>
-      <c r="D10" s="9"/>
+        <v>68</v>
+      </c>
+      <c r="D10" s="10"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" t="s">
         <v>57</v>
       </c>
-      <c r="B11" t="s">
-        <v>58</v>
-      </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" t="s">
         <v>59</v>
       </c>
-      <c r="B12" t="s">
-        <v>60</v>
-      </c>
       <c r="C12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" t="s">
         <v>61</v>
       </c>
-      <c r="B13" t="s">
-        <v>62</v>
-      </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" t="s">
         <v>63</v>
       </c>
-      <c r="B14" t="s">
-        <v>64</v>
-      </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>88</v>
+      <c r="A15" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>83</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1238,222 +1423,312 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="39.6640625" customWidth="1"/>
+    <col min="2" max="3" width="30.21875" customWidth="1"/>
+    <col min="4" max="4" width="39.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>42</v>
+        <v>116</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" s="14"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" s="14"/>
+    </row>
+    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B3" s="10" t="s">
+      <c r="B6" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="F3" s="13"/>
-    </row>
-    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="B4" s="10" t="s">
+      <c r="B7" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="F4" s="13"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
+      <c r="B12" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+      <c r="B14" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="10" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" s="10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" s="10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" s="10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="10" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A28" s="10" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" s="10" t="s">
-        <v>124</v>
+      <c r="B19" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:A4" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="1">
-    <mergeCell ref="F2:F4"/>
+    <mergeCell ref="D2:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1473,79 +1748,79 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1564,32 +1839,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cambios validaciones correo codigo antiguo para login vtex y ajustes c6
</commit_message>
<xml_diff>
--- a/data/ChedrahuiQA_Lexico.xlsx
+++ b/data/ChedrahuiQA_Lexico.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atcon\Desktop\Playwright\playwright-piloto2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D919A806-34FA-4ACB-9CB4-E95FE44062EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2909E0-1E33-4C81-A4C0-063F4E73EA3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Long Tail" sheetId="1" r:id="rId1"/>
-    <sheet name="Resultados vacíos" sheetId="2" r:id="rId2"/>
-    <sheet name="Errores Ortográficos" sheetId="3" r:id="rId3"/>
-    <sheet name="Frecuencia Alta" sheetId="4" r:id="rId4"/>
+    <sheet name="Contexto" sheetId="5" r:id="rId2"/>
+    <sheet name="Resultados vacíos" sheetId="2" r:id="rId3"/>
+    <sheet name="Errores Ortográficos" sheetId="3" r:id="rId4"/>
+    <sheet name="Frecuencia Alta" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="526">
   <si>
     <t>Término</t>
   </si>
@@ -1593,6 +1594,30 @@
   </si>
   <si>
     <t>Elotitos Tiernos</t>
+  </si>
+  <si>
+    <t>ingredientes para ceviche peruano</t>
+  </si>
+  <si>
+    <t>adorno para fiesta infantil</t>
+  </si>
+  <si>
+    <t>ingredientes pastel cumpleaños</t>
+  </si>
+  <si>
+    <t>cosas para ver peliculas</t>
+  </si>
+  <si>
+    <t>Limón, Pescado blanco, Cebolla morada, Ají limo, Cilantro, Sal, Pimienta, Camote, Choclo, Lechuga</t>
+  </si>
+  <si>
+    <t>Globos de colores, Banderines decorativos, guirnalda, Confeti, Mantel, Centro de Mesa, Velas, Piñata, Platos desechables, Servilletas decoradas</t>
+  </si>
+  <si>
+    <t>Harina, Huevos, Azucar, Mantequilla, Leche, Polvo para hornear, Vainilla, Crema para batir</t>
+  </si>
+  <si>
+    <t>Palomita de maiz, palomitas, pochoclo, refresco, nachos, queso para nachos, dulces, chocolate, papas, galletas, helado</t>
   </si>
 </sst>
 </file>
@@ -3023,6 +3048,60 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F33EBB3B-110B-4D61-81AB-57FEEF44EA94}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="45.6640625" customWidth="1"/>
+    <col min="2" max="2" width="118.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>518</v>
+      </c>
+      <c r="B2" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>519</v>
+      </c>
+      <c r="B3" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>520</v>
+      </c>
+      <c r="B4" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>521</v>
+      </c>
+      <c r="B5" t="s">
+        <v>525</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F034F82D-6CEA-4C71-B3F1-B7D6587367A8}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3201,7 +3280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E2ECB75-DF08-4ECD-8FCD-EE6E661D4C06}">
   <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3502,7 +3581,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64B01EF2-CEB5-4A1F-986E-1115CB160222}">
   <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>